<commit_message>
revised graph, text issue
</commit_message>
<xml_diff>
--- a/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
+++ b/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\oss\nietras.github.io\images\2025-06-sep-0.11.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84DE77E4-3767-4443-B1D2-1F04F8B6765F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED2A436-EC96-4E3A-92D2-8BD9903CDCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
   <si>
     <t>Sep</t>
   </si>
@@ -135,12 +135,6 @@
   </si>
   <si>
     <t>M1</t>
-  </si>
-  <si>
-    <t>Sep 0.6.0</t>
-  </si>
-  <si>
-    <t>Sep 0.9.0</t>
   </si>
   <si>
     <t>Sep 0.11.0</t>
@@ -908,7 +902,736 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.347140080786232E-2"/>
+          <c:y val="2.2553766250635515E-2"/>
+          <c:w val="0.87940287043705045"/>
+          <c:h val="0.87187278965479797"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$H$16</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>MB/s</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="2.3485982459176467E-2"/>
+                  <c:y val="-9.6658998217010531E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-9820-42EC-A8FC-E367FD3AF5BC}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="lt1">
+                        <a:lumMod val="85000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-DK"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="lt1">
+                          <a:lumMod val="95000"/>
+                          <a:alpha val="54000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$G$17:$G$20</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Sep 0.10.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sep 0.11.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Sylvan 1.4.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>CsvHelper 33.1.0</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$H$17:$H$20</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>6971.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9539.7000000000007</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="General">
+                  <c:v>1492</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>670.8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9820-42EC-A8FC-E367FD3AF5BC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="100"/>
+        <c:axId val="1489640399"/>
+        <c:axId val="1489638479"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$I$16</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Ratio</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="34925" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.5228973688764806E-2"/>
+                  <c:y val="3.866359928680374E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-9820-42EC-A8FC-E367FD3AF5BC}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.9143304098628283E-3"/>
+                  <c:y val="1.6109833036168194E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-9820-42EC-A8FC-E367FD3AF5BC}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.131464327890205E-2"/>
+                  <c:y val="3.866359928680374E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-9820-42EC-A8FC-E367FD3AF5BC}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-9.7858260246568921E-3"/>
+                  <c:y val="2.2553766250635515E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-9820-42EC-A8FC-E367FD3AF5BC}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="accent2"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-DK"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="lt1">
+                          <a:lumMod val="95000"/>
+                          <a:alpha val="54000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$G$17:$G$20</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Sep 0.10.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sep 0.11.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Sylvan 1.4.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>CsvHelper 33.1.0</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$I$17:$I$20</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>10.393261776982708</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14.221377459749554</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.2242098986285033</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9820-42EC-A8FC-E367FD3AF5BC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1369658991"/>
+        <c:axId val="1369653231"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1489640399"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-DK"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1489638479"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1489638479"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                  <a:alpha val="10000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-DK"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1489640399"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1369653231"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="18"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-DK"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1369658991"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="2"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="1369658991"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1369653231"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="1"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-DK"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="85000"/>
+        <a:lumOff val="15000"/>
+      </a:schemeClr>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-DK"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:userShapes r:id="rId3"/>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1444,20 +2167,516 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="34925" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>486604</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>160475</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>220465</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>6394</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>471073</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>204932</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>37272</xdr:rowOff>
+      <xdr:rowOff>65287</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1480,6 +2699,211 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>103707</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>146101</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>270699</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>81690</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D60AA3D-10F7-D370-255B-D6FCA817EFAB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>74707</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>149412</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>38205</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>93382</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB07A33D-4DC3-44EF-27B8-B2EE780F9A4B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3557869" y="4155515"/>
+          <a:ext cx="3208535" cy="1582831"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" rtlCol="0"/>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="3600" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Sep</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>World's Fastest .NET CSV</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> Parser</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2000" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Performance on </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="2000" u="sng" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Apple M1</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2000" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Progression and Comparison</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-DK" sz="1100" kern="1200">
+            <a:solidFill>
+              <a:srgbClr val="C198E0"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1626,6 +3050,49 @@
               <a:srgbClr val="C198E0"/>
             </a:solidFill>
           </a:endParaRPr>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+</c:userShapes>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.7453</cdr:x>
+      <cdr:y>0.50546</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.88621</cdr:x>
+      <cdr:y>0.73744</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39B48BE8-1A77-D246-FE5E-9B736EE9FD02}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="4836219" y="1992355"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-DK" sz="1100" kern="1200"/>
         </a:p>
       </cdr:txBody>
     </cdr:sp>
@@ -1896,7 +3363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -2345,72 +3812,48 @@
     </row>
     <row r="17" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H17" s="5">
-        <v>7732.9</v>
+        <v>6971.8</v>
       </c>
       <c r="I17" s="4">
-        <f t="shared" ref="I17:I20" si="1">H17/H$22</f>
-        <v>11.527877161598092</v>
+        <f>H17/H$20</f>
+        <v>10.393261776982708</v>
       </c>
     </row>
     <row r="18" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H18" s="5">
-        <v>7196.8</v>
+        <v>9539.7000000000007</v>
       </c>
       <c r="I18" s="4">
-        <f t="shared" si="1"/>
-        <v>10.728682170542637</v>
+        <f>H18/H$20</f>
+        <v>14.221377459749554</v>
       </c>
     </row>
     <row r="19" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G19" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="5">
-        <v>6971.8</v>
+        <v>35</v>
+      </c>
+      <c r="H19">
+        <v>1492</v>
       </c>
       <c r="I19" s="4">
-        <f t="shared" si="1"/>
-        <v>10.393261776982708</v>
+        <f>H19/H$20</f>
+        <v>2.2242098986285033</v>
       </c>
     </row>
     <row r="20" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H20" s="5">
-        <v>9539.7000000000007</v>
+        <v>670.8</v>
       </c>
       <c r="I20" s="4">
-        <f t="shared" si="1"/>
-        <v>14.221377459749554</v>
-      </c>
-    </row>
-    <row r="21" spans="7:9" x14ac:dyDescent="0.45">
-      <c r="G21" t="s">
-        <v>37</v>
-      </c>
-      <c r="H21">
-        <v>1492</v>
-      </c>
-      <c r="I21" s="4">
-        <f>H21/H$22</f>
-        <v>2.2242098986285033</v>
-      </c>
-    </row>
-    <row r="22" spans="7:9" x14ac:dyDescent="0.45">
-      <c r="G22" t="s">
-        <v>38</v>
-      </c>
-      <c r="H22" s="5">
-        <v>670.8</v>
-      </c>
-      <c r="I22" s="4">
         <f>1</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
add cobalt numbers to excel, fix in post
</commit_message>
<xml_diff>
--- a/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
+++ b/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\oss\nietras.github.io\images\2025-06-sep-0.11.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED2A436-EC96-4E3A-92D2-8BD9903CDCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C793E488-8178-4151-A7CD-E939774D8625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="38">
   <si>
     <t>Sep</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>CsvHelper 33.1.0</t>
+  </si>
+  <si>
+    <t>Cobalt 100</t>
   </si>
 </sst>
 </file>
@@ -1513,6 +1516,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1369653231"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3363,7 +3367,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -3810,7 +3814,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="7:9" x14ac:dyDescent="0.45">
+    <row r="17" spans="7:16" x14ac:dyDescent="0.45">
       <c r="G17" t="s">
         <v>34</v>
       </c>
@@ -3822,7 +3826,7 @@
         <v>10.393261776982708</v>
       </c>
     </row>
-    <row r="18" spans="7:9" x14ac:dyDescent="0.45">
+    <row r="18" spans="7:16" x14ac:dyDescent="0.45">
       <c r="G18" t="s">
         <v>33</v>
       </c>
@@ -3834,7 +3838,7 @@
         <v>14.221377459749554</v>
       </c>
     </row>
-    <row r="19" spans="7:9" x14ac:dyDescent="0.45">
+    <row r="19" spans="7:16" x14ac:dyDescent="0.45">
       <c r="G19" t="s">
         <v>35</v>
       </c>
@@ -3846,7 +3850,7 @@
         <v>2.2242098986285033</v>
       </c>
     </row>
-    <row r="20" spans="7:9" x14ac:dyDescent="0.45">
+    <row r="20" spans="7:16" x14ac:dyDescent="0.45">
       <c r="G20" t="s">
         <v>36</v>
       </c>
@@ -3854,6 +3858,70 @@
         <v>670.8</v>
       </c>
       <c r="I20" s="4">
+        <f>1</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="7:16" x14ac:dyDescent="0.45">
+      <c r="N22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="7:16" x14ac:dyDescent="0.45">
+      <c r="N23" t="s">
+        <v>31</v>
+      </c>
+      <c r="O23" t="s">
+        <v>16</v>
+      </c>
+      <c r="P23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="7:16" x14ac:dyDescent="0.45">
+      <c r="N24" t="s">
+        <v>34</v>
+      </c>
+      <c r="O24" s="5">
+        <v>3935</v>
+      </c>
+      <c r="P24" s="4">
+        <f>O24/O$27</f>
+        <v>7.0646319569120291</v>
+      </c>
+    </row>
+    <row r="25" spans="7:16" x14ac:dyDescent="0.45">
+      <c r="N25" t="s">
+        <v>33</v>
+      </c>
+      <c r="O25" s="5">
+        <v>6117</v>
+      </c>
+      <c r="P25" s="4">
+        <f>O25/O$27</f>
+        <v>10.982046678635548</v>
+      </c>
+    </row>
+    <row r="26" spans="7:16" x14ac:dyDescent="0.45">
+      <c r="N26" t="s">
+        <v>35</v>
+      </c>
+      <c r="O26">
+        <v>1461</v>
+      </c>
+      <c r="P26" s="4">
+        <f>O26/O$27</f>
+        <v>2.6229802513464993</v>
+      </c>
+    </row>
+    <row r="27" spans="7:16" x14ac:dyDescent="0.45">
+      <c r="N27" t="s">
+        <v>36</v>
+      </c>
+      <c r="O27" s="5">
+        <v>557</v>
+      </c>
+      <c r="P27" s="4">
         <f>1</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
fix chart for apple m1 with extra text
</commit_message>
<xml_diff>
--- a/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
+++ b/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\oss\nietras.github.io\images\2025-06-sep-0.11.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\oss\nietras.github.io\images\2025-06-sep-0.11.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C793E488-8178-4151-A7CD-E939774D8625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324C8917-9E86-48D1-B57F-4DC0252ADE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -207,9 +207,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FF7CAFDE"/>
       <color rgb="FFC198E0"/>
       <color rgb="FFB482DA"/>
+      <color rgb="FF7CAFDE"/>
     </mruColors>
   </colors>
   <extLst>
@@ -2741,175 +2741,6 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>74707</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>149412</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>38205</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>93382</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB07A33D-4DC3-44EF-27B8-B2EE780F9A4B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3557869" y="4155515"/>
-          <a:ext cx="3208535" cy="1582831"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0"/>
-        <a:lstStyle>
-          <a:lvl1pPr marL="0" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="3600" kern="1200">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Sep</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400" kern="1200">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>World's Fastest .NET CSV</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t> Parser</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Performance on </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" u="sng" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Apple M1</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Progression and Comparison</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-DK" sz="1100" kern="1200">
-            <a:solidFill>
-              <a:srgbClr val="C198E0"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3097,6 +2928,202 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:endParaRPr lang="en-DK" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.42366</cdr:x>
+      <cdr:y>0</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>1</cdr:x>
+      <cdr:y>0.66219</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3992948E-522E-3392-DA69-61D77987F653}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="2749124" y="0"/>
+          <a:ext cx="3739853" cy="2610142"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="square" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr kumimoji="0" lang="en-US" sz="3600" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0" noProof="0">
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uLnTx/>
+              <a:uFillTx/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Sep</a:t>
+          </a:r>
+        </a:p>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr kumimoji="0" lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0" noProof="0">
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uLnTx/>
+              <a:uFillTx/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>World's Fastest .NET CSV Parser</a:t>
+          </a:r>
+        </a:p>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr kumimoji="0" lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0" noProof="0">
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uLnTx/>
+              <a:uFillTx/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Performance Progression and Comparison on</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr kumimoji="0" lang="en-US" sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0" noProof="0">
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uLnTx/>
+              <a:uFillTx/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+        </a:p>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr kumimoji="0" lang="en-US" sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0" noProof="0">
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C198E0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uLnTx/>
+              <a:uFillTx/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Apple M1</a:t>
+          </a:r>
         </a:p>
       </cdr:txBody>
     </cdr:sp>

</xml_diff>

<commit_message>
add cobalt 100 chart
</commit_message>
<xml_diff>
--- a/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
+++ b/images/2025-06-sep-0.11.0/sep-perf-0.11.0-apple-m1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\oss\nietras.github.io\images\2025-06-sep-0.11.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324C8917-9E86-48D1-B57F-4DC0252ADE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9DED07E-4290-433A-AEAF-73FA38D8CB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -224,688 +224,6 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="5.7769752498476178E-2"/>
-          <c:y val="3.1430158846042958E-2"/>
-          <c:w val="0.87161199067706208"/>
-          <c:h val="0.82411320136791311"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$H$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>MB/s</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent1">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent1">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dPt>
-            <c:idx val="10"/>
-            <c:invertIfNegative val="0"/>
-            <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="92D050"/>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst>
-                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                  <a:srgbClr val="000000">
-                    <a:alpha val="63000"/>
-                  </a:srgbClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </c:spPr>
-            <c:extLst>
-              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000000-7927-4577-9AB4-0FCBAA089B2C}"/>
-              </c:ext>
-            </c:extLst>
-          </c:dPt>
-          <c:dPt>
-            <c:idx val="11"/>
-            <c:invertIfNegative val="0"/>
-            <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="92D050"/>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst>
-                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                  <a:srgbClr val="000000">
-                    <a:alpha val="63000"/>
-                  </a:srgbClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </c:spPr>
-            <c:extLst>
-              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-7927-4577-9AB4-0FCBAA089B2C}"/>
-              </c:ext>
-            </c:extLst>
-          </c:dPt>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="bg2"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-DK"/>
-              </a:p>
-            </c:txPr>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </c15:spPr>
-                <c15:showLeaderLines val="0"/>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$D$2:$D$13</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>Sep 0.1.0, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Sep 0.2.0, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Sep 0.2.1, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Sep 0.3.0, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Sep 0.3.0, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Sep 0.4.0, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Sep 0.4.1, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Sep 0.5.0, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Sep 0.6.0, .NET 9.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Sep 0.9.0, .NET 9.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Sep 0.9.0, .NET 9.0, 9950X </c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Sep 0.10.0, .NET 9.0, 9950X</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$H$2:$H$13</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>7335.3</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>10191.6</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>11120.2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>11503.7</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>12111.6</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>12581.3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>12811.2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>12544.5</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>13339.9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>13088.4</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>18202.7</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>21384.9</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FFE8-4851-9A7D-1D421F82BD55}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="100"/>
-        <c:overlap val="-24"/>
-        <c:axId val="973515696"/>
-        <c:axId val="973499376"/>
-      </c:barChart>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$J$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Ratio</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="34925" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$D$2:$D$13</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>Sep 0.1.0, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Sep 0.2.0, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Sep 0.2.1, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Sep 0.3.0, .NET 7.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Sep 0.3.0, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Sep 0.4.0, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Sep 0.4.1, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Sep 0.5.0, .NET 8.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Sep 0.6.0, .NET 9.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Sep 0.9.0, .NET 9.0, 5950X </c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Sep 0.9.0, .NET 9.0, 9950X </c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Sep 0.10.0, .NET 9.0, 9950X</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$J$2:$J$13</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.389391026951863</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.5159843496516845</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.5682657832672147</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.6511390127193162</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.7151718402791978</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.746513435033332</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.7101550038853217</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.8185895600725259</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.784303300478508</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>2.4815208648589695</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>2.9153408858533396</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-FFE8-4851-9A7D-1D421F82BD55}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="974443600"/>
-        <c:axId val="974442640"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="973515696"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="lt1">
-                <a:lumMod val="95000"/>
-                <a:alpha val="54000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-DK"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="973499376"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="973499376"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="95000"/>
-                  <a:alpha val="10000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-DK"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="973515696"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="974442640"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="r"/>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-DK"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="974443600"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:catAx>
-        <c:axId val="974443600"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="974442640"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="8.700024893218232E-2"/>
-          <c:y val="6.2263744988530059E-2"/>
-          <c:w val="0.16734367396867736"/>
-          <c:h val="0.11994759484797152"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-DK"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="tx1">
-        <a:lumMod val="85000"/>
-        <a:lumOff val="15000"/>
-      </a:schemeClr>
-    </a:solidFill>
-    <a:ln>
-      <a:noFill/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-DK"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-  <c:userShapes r:id="rId3"/>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1092,16 +410,16 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>6971.8</c:v>
+                  <c:v>3935</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9539.7000000000007</c:v>
+                  <c:v>6117</c:v>
                 </c:pt>
                 <c:pt idx="2" formatCode="General">
-                  <c:v>1492</c:v>
+                  <c:v>1461</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>670.8</c:v>
+                  <c:v>557</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1323,13 +641,13 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>10.393261776982708</c:v>
+                  <c:v>7.0646319569120291</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14.221377459749554</c:v>
+                  <c:v>10.982046678635548</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.2242098986285033</c:v>
+                  <c:v>2.6229802513464993</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>1</c:v>
@@ -1411,6 +729,7 @@
         <c:axId val="1489638479"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="8000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1464,7 +783,7 @@
         <c:axId val="1369653231"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="18"/>
+          <c:max val="14.4"/>
           <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -1635,46 +954,6 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
   <cs:axisTitle>
@@ -2171,540 +1450,8 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:gradFill flip="none" rotWithShape="1">
-        <a:gsLst>
-          <a:gs pos="0">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="65000"/>
-              <a:lumOff val="35000"/>
-            </a:schemeClr>
-          </a:gs>
-          <a:gs pos="100000">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="85000"/>
-              <a:lumOff val="15000"/>
-            </a:schemeClr>
-          </a:gs>
-        </a:gsLst>
-        <a:path path="circle">
-          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-        </a:path>
-        <a:tileRect/>
-      </a:gradFill>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="34925" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="10000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="5000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="95000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
-      <a:effectLst>
-        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-          <a:prstClr val="black">
-            <a:alpha val="40000"/>
-          </a:prstClr>
-        </a:outerShdw>
-      </a:effectLst>
-    </cs:defRPr>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>220465</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>6394</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>204932</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>65287</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80A60280-E58C-B6DA-EC09-A2A64346C53B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -2735,7 +1482,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2745,154 +1492,6 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.7828</cdr:x>
-      <cdr:y>0</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.78499</cdr:x>
-      <cdr:y>1</cdr:y>
-    </cdr:to>
-    <cdr:cxnSp macro="">
-      <cdr:nvCxnSpPr>
-        <cdr:cNvPr id="3" name="Straight Connector 2">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DA92422-2B5F-8441-9152-04C287BCECF4}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvCxnSpPr/>
-      </cdr:nvCxnSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" flipH="1">
-          <a:off x="5559700" y="0"/>
-          <a:ext cx="15530" cy="4949895"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="15875">
-          <a:solidFill>
-            <a:srgbClr val="FFFF00"/>
-          </a:solidFill>
-          <a:prstDash val="dash"/>
-        </a:ln>
-      </cdr:spPr>
-      <cdr:style>
-        <a:lnRef xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </cdr:style>
-    </cdr:cxnSp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.29446</cdr:x>
-      <cdr:y>0.02196</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.7121</cdr:x>
-      <cdr:y>0.34616</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF858AA7-EB79-0A01-540A-6CCBAFA5FEC8}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="2091354" y="108699"/>
-          <a:ext cx="2966219" cy="1604765"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="3600" kern="1200">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Sep</a:t>
-          </a:r>
-        </a:p>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400" kern="1200">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>World's Fastest .NET CSV</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t> Parser</a:t>
-          </a:r>
-        </a:p>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Performance on Apple M1</a:t>
-          </a:r>
-        </a:p>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="C198E0"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Progression and Comparison</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-DK" sz="1100" kern="1200">
-            <a:solidFill>
-              <a:srgbClr val="C198E0"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-</c:userShapes>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
@@ -3846,11 +2445,11 @@
         <v>34</v>
       </c>
       <c r="H17" s="5">
-        <v>6971.8</v>
+        <v>3935</v>
       </c>
       <c r="I17" s="4">
         <f>H17/H$20</f>
-        <v>10.393261776982708</v>
+        <v>7.0646319569120291</v>
       </c>
     </row>
     <row r="18" spans="7:16" x14ac:dyDescent="0.45">
@@ -3858,11 +2457,11 @@
         <v>33</v>
       </c>
       <c r="H18" s="5">
-        <v>9539.7000000000007</v>
+        <v>6117</v>
       </c>
       <c r="I18" s="4">
         <f>H18/H$20</f>
-        <v>14.221377459749554</v>
+        <v>10.982046678635548</v>
       </c>
     </row>
     <row r="19" spans="7:16" x14ac:dyDescent="0.45">
@@ -3870,11 +2469,11 @@
         <v>35</v>
       </c>
       <c r="H19">
-        <v>1492</v>
+        <v>1461</v>
       </c>
       <c r="I19" s="4">
         <f>H19/H$20</f>
-        <v>2.2242098986285033</v>
+        <v>2.6229802513464993</v>
       </c>
     </row>
     <row r="20" spans="7:16" x14ac:dyDescent="0.45">
@@ -3882,7 +2481,7 @@
         <v>36</v>
       </c>
       <c r="H20" s="5">
-        <v>670.8</v>
+        <v>557</v>
       </c>
       <c r="I20" s="4">
         <f>1</f>

</xml_diff>